<commit_message>
Updated TJK_grids model - 2025-09-25 14:13
</commit_message>
<xml_diff>
--- a/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_TJK_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{674BE192-11A7-4D77-8D79-DF0329E6E917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{235F4A91-30E1-45D8-86C8-783ADF27B2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -771,6 +771,18 @@
     <t>daynite</t>
   </si>
   <si>
+    <t>distr_solelc_spv_010</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_007</t>
   </si>
   <si>
@@ -783,42 +795,30 @@
     <t>connecting solar to buses in cluster 2</t>
   </si>
   <si>
+    <t>distr_solelc_spv_006</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_009</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 9</t>
   </si>
   <si>
-    <t>distr_solelc_spv_006</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_010</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_001</t>
   </si>
   <si>
@@ -834,30 +834,30 @@
     <t>e_w1373384046-500,e_w1016951696-500,e_w799346816-500</t>
   </si>
   <si>
+    <t>e_TJ30-500,e_w242159365-500,e_TJ26-500</t>
+  </si>
+  <si>
+    <t>e_w1373384046-500</t>
+  </si>
+  <si>
     <t>e_w799346816-500,e_TJ26-500,e_TJ10-500</t>
   </si>
   <si>
     <t>e_TJ10-500</t>
   </si>
   <si>
+    <t>e_TJ46-500,e_w1373384046-500</t>
+  </si>
+  <si>
+    <t>e_TJ46-500,e_w488077624-500</t>
+  </si>
+  <si>
+    <t>e_TJ20-500,e_TJ6-500,e_TJ26-500,e_TJ4-500,e_TJ10-500</t>
+  </si>
+  <si>
     <t>e_w488077624-500,e_TJ20-500</t>
   </si>
   <si>
-    <t>e_TJ46-500,e_w1373384046-500</t>
-  </si>
-  <si>
-    <t>e_TJ46-500,e_w488077624-500</t>
-  </si>
-  <si>
-    <t>e_TJ20-500,e_TJ6-500,e_TJ26-500,e_TJ4-500,e_TJ10-500</t>
-  </si>
-  <si>
-    <t>e_TJ30-500,e_w242159365-500,e_TJ26-500</t>
-  </si>
-  <si>
-    <t>e_w1373384046-500</t>
-  </si>
-  <si>
     <t>e_w799346816-500</t>
   </si>
   <si>
@@ -879,18 +879,18 @@
     <t>connecting wind onshore to buses in cluster 5</t>
   </si>
   <si>
+    <t>distr_wonelc_won_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_004</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 4</t>
   </si>
   <si>
-    <t>distr_wonelc_won_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
     <t>elc_won_002</t>
   </si>
   <si>
@@ -903,16 +903,16 @@
     <t>elc_won_005</t>
   </si>
   <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>e_TJ6-500</t>
+  </si>
+  <si>
     <t>elc_won_004</t>
   </si>
   <si>
     <t>e_TJ4-500</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>e_TJ6-500</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -5721,7 +5721,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC38DF7-AC7F-480A-9A96-F3375A7593B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B5E8F92-DE68-4547-AD88-FF48358E982D}">
   <dimension ref="B9:AP20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -5956,7 +5956,7 @@
         <v>254</v>
       </c>
       <c r="AN11" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="AO11">
         <v>0.9927360267512606</v>
@@ -6027,16 +6027,16 @@
         <v>214</v>
       </c>
       <c r="Y12" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="Z12" t="s">
         <v>235</v>
       </c>
       <c r="AA12">
-        <v>0.99559026704960707</v>
+        <v>0.9973662353879873</v>
       </c>
       <c r="AB12">
-        <v>80.845104090536353</v>
+        <v>48.285684553565716</v>
       </c>
       <c r="AD12" t="s">
         <v>209</v>
@@ -6137,16 +6137,16 @@
         <v>216</v>
       </c>
       <c r="Y13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="Z13" t="s">
         <v>236</v>
       </c>
       <c r="AA13">
-        <v>0.99727051178070425</v>
+        <v>0.99508741713487281</v>
       </c>
       <c r="AB13">
-        <v>50.040617353755373</v>
+        <v>90.064019193998561</v>
       </c>
       <c r="AD13" t="s">
         <v>209</v>
@@ -6176,7 +6176,7 @@
         <v>257</v>
       </c>
       <c r="AN13" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AO13">
         <v>0.99763776609661003</v>
@@ -6247,16 +6247,16 @@
         <v>218</v>
       </c>
       <c r="Y14" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="Z14" t="s">
         <v>237</v>
       </c>
       <c r="AA14">
-        <v>0.99510391360728279</v>
+        <v>0.99559026704960707</v>
       </c>
       <c r="AB14">
-        <v>89.761583866481658</v>
+        <v>80.845104090536353</v>
       </c>
       <c r="AD14" t="s">
         <v>209</v>
@@ -6289,10 +6289,10 @@
         <v>259</v>
       </c>
       <c r="AO14">
-        <v>0.99832227355557335</v>
+        <v>0.99828324379345523</v>
       </c>
       <c r="AP14">
-        <v>30.758318147821576</v>
+        <v>31.473863786654263</v>
       </c>
     </row>
     <row r="15" spans="2:42">
@@ -6357,16 +6357,16 @@
         <v>220</v>
       </c>
       <c r="Y15" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="Z15" t="s">
         <v>238</v>
       </c>
       <c r="AA15">
-        <v>0.99483713382754202</v>
+        <v>0.99727051178070425</v>
       </c>
       <c r="AB15">
-        <v>94.652546495062282</v>
+        <v>50.040617353755373</v>
       </c>
       <c r="AD15" t="s">
         <v>209</v>
@@ -6399,10 +6399,10 @@
         <v>261</v>
       </c>
       <c r="AO15">
-        <v>0.99828324379345523</v>
+        <v>0.99832227355557335</v>
       </c>
       <c r="AP15">
-        <v>31.473863786654263</v>
+        <v>30.758318147821576</v>
       </c>
     </row>
     <row r="16" spans="2:42">
@@ -6467,16 +6467,16 @@
         <v>222</v>
       </c>
       <c r="Y16" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="Z16" t="s">
         <v>239</v>
       </c>
       <c r="AA16">
-        <v>0.9966237176926277</v>
+        <v>0.99483713382754202</v>
       </c>
       <c r="AB16">
-        <v>61.898508968492948</v>
+        <v>94.652546495062282</v>
       </c>
     </row>
     <row r="17" spans="2:28">
@@ -6541,16 +6541,16 @@
         <v>224</v>
       </c>
       <c r="Y17" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="Z17" t="s">
         <v>240</v>
       </c>
       <c r="AA17">
-        <v>0.99797437485078455</v>
+        <v>0.9966237176926277</v>
       </c>
       <c r="AB17">
-        <v>37.136461068950517</v>
+        <v>61.898508968492948</v>
       </c>
     </row>
     <row r="18" spans="2:28">
@@ -6615,16 +6615,16 @@
         <v>226</v>
       </c>
       <c r="Y18" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="Z18" t="s">
         <v>241</v>
       </c>
       <c r="AA18">
-        <v>0.9973662353879873</v>
+        <v>0.99797437485078455</v>
       </c>
       <c r="AB18">
-        <v>48.285684553565716</v>
+        <v>37.136461068950517</v>
       </c>
     </row>
     <row r="19" spans="2:28">
@@ -6689,16 +6689,16 @@
         <v>228</v>
       </c>
       <c r="Y19" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="Z19" t="s">
         <v>242</v>
       </c>
       <c r="AA19">
-        <v>0.99508741713487281</v>
+        <v>0.99510391360728279</v>
       </c>
       <c r="AB19">
-        <v>90.064019193998561</v>
+        <v>89.761583866481658</v>
       </c>
     </row>
     <row r="20" spans="2:28">
@@ -6781,7 +6781,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDED94AB-0798-47DD-83FE-EA22C4F01314}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E902210F-4D73-40A9-BB96-9C708C4D4AF2}">
   <dimension ref="B9:M15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6924,7 +6924,7 @@
         <v>266</v>
       </c>
       <c r="K13" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L13">
         <v>1.2619807953067491E-2</v>
@@ -6959,7 +6959,7 @@
         <v>268</v>
       </c>
       <c r="K14" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L14">
         <v>0.43107241214667685</v>
@@ -7009,7 +7009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0754AB46-62AA-4175-90DD-1DEDA7C7BF89}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4A9789-FBC4-4C27-BD9B-D686FF3F531E}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated TJK_grids model - 2025-09-25 14:17
</commit_message>
<xml_diff>
--- a/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_TJK_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{235F4A91-30E1-45D8-86C8-783ADF27B2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD89D1B5-0ADB-4002-8BAC-E4738A9B5897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -759,16 +759,40 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_006</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_004</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_003</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 3</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
+    <t>distr_solelc_spv_001</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 1</t>
   </si>
   <si>
     <t>distr_solelc_spv_010</t>
@@ -783,6 +807,12 @@
     <t>connecting solar to buses in cluster 5</t>
   </si>
   <si>
+    <t>distr_solelc_spv_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_007</t>
   </si>
   <si>
@@ -795,70 +825,58 @@
     <t>connecting solar to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_solelc_spv_006</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_004</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_001</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 1</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_TJ46-500,e_w1373384046-500</t>
+  </si>
+  <si>
+    <t>e_TJ46-500,e_w488077624-500</t>
+  </si>
+  <si>
+    <t>e_TJ20-500,e_TJ6-500,e_TJ26-500,e_TJ4-500,e_TJ10-500</t>
+  </si>
+  <si>
     <t>e_w1373384046-500,e_w1016951696-500,e_w799346816-500</t>
   </si>
   <si>
+    <t>e_w799346816-500</t>
+  </si>
+  <si>
     <t>e_TJ30-500,e_w242159365-500,e_TJ26-500</t>
   </si>
   <si>
     <t>e_w1373384046-500</t>
   </si>
   <si>
+    <t>e_w488077624-500,e_TJ20-500</t>
+  </si>
+  <si>
     <t>e_w799346816-500,e_TJ26-500,e_TJ10-500</t>
   </si>
   <si>
     <t>e_TJ10-500</t>
   </si>
   <si>
-    <t>e_TJ46-500,e_w1373384046-500</t>
-  </si>
-  <si>
-    <t>e_TJ46-500,e_w488077624-500</t>
-  </si>
-  <si>
-    <t>e_TJ20-500,e_TJ6-500,e_TJ26-500,e_TJ4-500,e_TJ10-500</t>
-  </si>
-  <si>
-    <t>e_w488077624-500,e_TJ20-500</t>
-  </si>
-  <si>
-    <t>e_w799346816-500</t>
+    <t>distr_wonelc_won_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_005</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 5</t>
   </si>
   <si>
     <t>distr_wonelc_won_002</t>
@@ -867,52 +885,34 @@
     <t>connecting wind onshore to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_wonelc_won_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_005</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 5</t>
-  </si>
-  <si>
     <t>distr_wonelc_won_003</t>
   </si>
   <si>
     <t>connecting wind onshore to buses in cluster 3</t>
   </si>
   <si>
-    <t>distr_wonelc_won_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>e_TJ4-500</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>e_TJ46-500</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
   </si>
   <si>
     <t>elc_won_002</t>
   </si>
   <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>e_TJ46-500</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
     <t>elc_won_003</t>
   </si>
   <si>
     <t>e_TJ6-500</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>e_TJ4-500</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -5721,7 +5721,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B5E8F92-DE68-4547-AD88-FF48358E982D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA24729-660A-40C6-9A85-7A0B1C003BF5}">
   <dimension ref="B9:AP20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -5917,16 +5917,16 @@
         <v>210</v>
       </c>
       <c r="Y11" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z11" t="s">
         <v>234</v>
       </c>
       <c r="AA11">
-        <v>0.998201681747511</v>
+        <v>0.99483713382754202</v>
       </c>
       <c r="AB11">
-        <v>32.969167962298094</v>
+        <v>94.652546495062282</v>
       </c>
       <c r="AD11" t="s">
         <v>209</v>
@@ -5956,13 +5956,13 @@
         <v>254</v>
       </c>
       <c r="AN11" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
       <c r="AO11">
-        <v>0.9927360267512606</v>
+        <v>0.99832227355557335</v>
       </c>
       <c r="AP11">
-        <v>133.17284289355615</v>
+        <v>30.758318147821576</v>
       </c>
     </row>
     <row r="12" spans="2:42">
@@ -6027,16 +6027,16 @@
         <v>214</v>
       </c>
       <c r="Y12" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="Z12" t="s">
         <v>235</v>
       </c>
       <c r="AA12">
-        <v>0.9973662353879873</v>
+        <v>0.9966237176926277</v>
       </c>
       <c r="AB12">
-        <v>48.285684553565716</v>
+        <v>61.898508968492948</v>
       </c>
       <c r="AD12" t="s">
         <v>209</v>
@@ -6063,10 +6063,10 @@
         <v>246</v>
       </c>
       <c r="AM12" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AN12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AO12">
         <v>0.99545389931512118</v>
@@ -6137,16 +6137,16 @@
         <v>216</v>
       </c>
       <c r="Y13" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="Z13" t="s">
         <v>236</v>
       </c>
       <c r="AA13">
-        <v>0.99508741713487281</v>
+        <v>0.99797437485078455</v>
       </c>
       <c r="AB13">
-        <v>90.064019193998561</v>
+        <v>37.136461068950517</v>
       </c>
       <c r="AD13" t="s">
         <v>209</v>
@@ -6173,10 +6173,10 @@
         <v>248</v>
       </c>
       <c r="AM13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AN13" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="AO13">
         <v>0.99763776609661003</v>
@@ -6247,16 +6247,16 @@
         <v>218</v>
       </c>
       <c r="Y14" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="Z14" t="s">
         <v>237</v>
       </c>
       <c r="AA14">
-        <v>0.99559026704960707</v>
+        <v>0.998201681747511</v>
       </c>
       <c r="AB14">
-        <v>80.845104090536353</v>
+        <v>32.969167962298094</v>
       </c>
       <c r="AD14" t="s">
         <v>209</v>
@@ -6283,16 +6283,16 @@
         <v>250</v>
       </c>
       <c r="AM14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AN14" t="s">
-        <v>259</v>
+        <v>240</v>
       </c>
       <c r="AO14">
-        <v>0.99828324379345523</v>
+        <v>0.9927360267512606</v>
       </c>
       <c r="AP14">
-        <v>31.473863786654263</v>
+        <v>133.17284289355615</v>
       </c>
     </row>
     <row r="15" spans="2:42">
@@ -6357,16 +6357,16 @@
         <v>220</v>
       </c>
       <c r="Y15" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Z15" t="s">
         <v>238</v>
       </c>
       <c r="AA15">
-        <v>0.99727051178070425</v>
+        <v>0.98763915166972838</v>
       </c>
       <c r="AB15">
-        <v>50.040617353755373</v>
+        <v>226.61555272164699</v>
       </c>
       <c r="AD15" t="s">
         <v>209</v>
@@ -6399,10 +6399,10 @@
         <v>261</v>
       </c>
       <c r="AO15">
-        <v>0.99832227355557335</v>
+        <v>0.99828324379345523</v>
       </c>
       <c r="AP15">
-        <v>30.758318147821576</v>
+        <v>31.473863786654263</v>
       </c>
     </row>
     <row r="16" spans="2:42">
@@ -6467,16 +6467,16 @@
         <v>222</v>
       </c>
       <c r="Y16" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="Z16" t="s">
         <v>239</v>
       </c>
       <c r="AA16">
-        <v>0.99483713382754202</v>
+        <v>0.9973662353879873</v>
       </c>
       <c r="AB16">
-        <v>94.652546495062282</v>
+        <v>48.285684553565716</v>
       </c>
     </row>
     <row r="17" spans="2:28">
@@ -6541,16 +6541,16 @@
         <v>224</v>
       </c>
       <c r="Y17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="Z17" t="s">
         <v>240</v>
       </c>
       <c r="AA17">
-        <v>0.9966237176926277</v>
+        <v>0.99508741713487281</v>
       </c>
       <c r="AB17">
-        <v>61.898508968492948</v>
+        <v>90.064019193998561</v>
       </c>
     </row>
     <row r="18" spans="2:28">
@@ -6615,16 +6615,16 @@
         <v>226</v>
       </c>
       <c r="Y18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Z18" t="s">
         <v>241</v>
       </c>
       <c r="AA18">
-        <v>0.99797437485078455</v>
+        <v>0.99510391360728279</v>
       </c>
       <c r="AB18">
-        <v>37.136461068950517</v>
+        <v>89.761583866481658</v>
       </c>
     </row>
     <row r="19" spans="2:28">
@@ -6689,16 +6689,16 @@
         <v>228</v>
       </c>
       <c r="Y19" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="Z19" t="s">
         <v>242</v>
       </c>
       <c r="AA19">
-        <v>0.99510391360728279</v>
+        <v>0.99559026704960707</v>
       </c>
       <c r="AB19">
-        <v>89.761583866481658</v>
+        <v>80.845104090536353</v>
       </c>
     </row>
     <row r="20" spans="2:28">
@@ -6763,16 +6763,16 @@
         <v>230</v>
       </c>
       <c r="Y20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Z20" t="s">
         <v>243</v>
       </c>
       <c r="AA20">
-        <v>0.98763915166972838</v>
+        <v>0.99727051178070425</v>
       </c>
       <c r="AB20">
-        <v>226.61555272164699</v>
+        <v>50.040617353755373</v>
       </c>
     </row>
   </sheetData>
@@ -6781,7 +6781,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E902210F-4D73-40A9-BB96-9C708C4D4AF2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F685A0A5-7E95-4D42-84DB-CC8F3801B256}">
   <dimension ref="B9:M15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6854,7 +6854,7 @@
         <v>262</v>
       </c>
       <c r="K11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L11">
         <v>1.2897218124341414</v>
@@ -6889,7 +6889,7 @@
         <v>264</v>
       </c>
       <c r="K12" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="L12">
         <v>0.28038164602463972</v>
@@ -6924,7 +6924,7 @@
         <v>266</v>
       </c>
       <c r="K13" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L13">
         <v>1.2619807953067491E-2</v>
@@ -6959,7 +6959,7 @@
         <v>268</v>
       </c>
       <c r="K14" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="L14">
         <v>0.43107241214667685</v>
@@ -6994,7 +6994,7 @@
         <v>270</v>
       </c>
       <c r="K15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L15">
         <v>0.22221482050297564</v>
@@ -7009,7 +7009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4A9789-FBC4-4C27-BD9B-D686FF3F531E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87773F4C-678B-4309-BEC1-C5C693AD9153}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated TJK_grids model - 2025-09-25 15:21
</commit_message>
<xml_diff>
--- a/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_TJK_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_TJK_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD89D1B5-0ADB-4002-8BAC-E4738A9B5897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{396B0CE9-2431-4F58-86FC-640BEA14E38B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -759,18 +759,42 @@
     <t>pre</t>
   </si>
   <si>
+    <t>distr_solelc_spv_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>NRGI</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_007</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_002</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_006</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 6</t>
   </si>
   <si>
-    <t>NRGI</t>
-  </si>
-  <si>
-    <t>daynite</t>
-  </si>
-  <si>
     <t>distr_solelc_spv_004</t>
   </si>
   <si>
@@ -783,10 +807,16 @@
     <t>connecting solar to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_solelc_spv_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
+    <t>distr_solelc_spv_010</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 10</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
   </si>
   <si>
     <t>distr_solelc_spv_001</t>
@@ -795,42 +825,24 @@
     <t>connecting solar to buses in cluster 1</t>
   </si>
   <si>
-    <t>distr_solelc_spv_010</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_007</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 7</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_002</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 2</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
     <t>ncap_cost~USD21_alt</t>
   </si>
   <si>
+    <t>e_w1373384046-500,e_w1016951696-500,e_w799346816-500</t>
+  </si>
+  <si>
+    <t>e_w799346816-500,e_TJ26-500,e_TJ10-500</t>
+  </si>
+  <si>
+    <t>e_TJ10-500</t>
+  </si>
+  <si>
+    <t>e_w488077624-500,e_TJ20-500</t>
+  </si>
+  <si>
     <t>e_TJ46-500,e_w1373384046-500</t>
   </si>
   <si>
@@ -840,25 +852,19 @@
     <t>e_TJ20-500,e_TJ6-500,e_TJ26-500,e_TJ4-500,e_TJ10-500</t>
   </si>
   <si>
-    <t>e_w1373384046-500,e_w1016951696-500,e_w799346816-500</t>
+    <t>e_TJ30-500,e_w242159365-500,e_TJ26-500</t>
+  </si>
+  <si>
+    <t>e_w1373384046-500</t>
   </si>
   <si>
     <t>e_w799346816-500</t>
   </si>
   <si>
-    <t>e_TJ30-500,e_w242159365-500,e_TJ26-500</t>
-  </si>
-  <si>
-    <t>e_w1373384046-500</t>
-  </si>
-  <si>
-    <t>e_w488077624-500,e_TJ20-500</t>
-  </si>
-  <si>
-    <t>e_w799346816-500,e_TJ26-500,e_TJ10-500</t>
-  </si>
-  <si>
-    <t>e_TJ10-500</t>
+    <t>distr_wonelc_won_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
   </si>
   <si>
     <t>distr_wonelc_won_004</t>
@@ -867,6 +873,12 @@
     <t>connecting wind onshore to buses in cluster 4</t>
   </si>
   <si>
+    <t>distr_wonelc_won_002</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 2</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_001</t>
   </si>
   <si>
@@ -879,16 +891,10 @@
     <t>connecting wind onshore to buses in cluster 5</t>
   </si>
   <si>
-    <t>distr_wonelc_won_002</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>e_TJ6-500</t>
   </si>
   <si>
     <t>elc_won_004</t>
@@ -897,6 +903,9 @@
     <t>e_TJ4-500</t>
   </si>
   <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
     <t>elc_won_001</t>
   </si>
   <si>
@@ -904,15 +913,6 @@
   </si>
   <si>
     <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>e_TJ6-500</t>
   </si>
   <si>
     <t>e_won_001</t>
@@ -5721,7 +5721,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA24729-660A-40C6-9A85-7A0B1C003BF5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E550AEDD-E781-4D32-8A17-BEDD09E2C07C}">
   <dimension ref="B9:AP20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -5917,16 +5917,16 @@
         <v>210</v>
       </c>
       <c r="Y11" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="Z11" t="s">
         <v>234</v>
       </c>
       <c r="AA11">
-        <v>0.99483713382754202</v>
+        <v>0.998201681747511</v>
       </c>
       <c r="AB11">
-        <v>94.652546495062282</v>
+        <v>32.969167962298094</v>
       </c>
       <c r="AD11" t="s">
         <v>209</v>
@@ -5959,10 +5959,10 @@
         <v>255</v>
       </c>
       <c r="AO11">
-        <v>0.99832227355557335</v>
+        <v>0.99828324379345523</v>
       </c>
       <c r="AP11">
-        <v>30.758318147821576</v>
+        <v>31.473863786654263</v>
       </c>
     </row>
     <row r="12" spans="2:42">
@@ -6027,16 +6027,16 @@
         <v>214</v>
       </c>
       <c r="Y12" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="Z12" t="s">
         <v>235</v>
       </c>
       <c r="AA12">
-        <v>0.9966237176926277</v>
+        <v>0.99559026704960707</v>
       </c>
       <c r="AB12">
-        <v>61.898508968492948</v>
+        <v>80.845104090536353</v>
       </c>
       <c r="AD12" t="s">
         <v>209</v>
@@ -6069,10 +6069,10 @@
         <v>257</v>
       </c>
       <c r="AO12">
-        <v>0.99545389931512118</v>
+        <v>0.99832227355557335</v>
       </c>
       <c r="AP12">
-        <v>83.345179222779151</v>
+        <v>30.758318147821576</v>
       </c>
     </row>
     <row r="13" spans="2:42">
@@ -6137,16 +6137,16 @@
         <v>216</v>
       </c>
       <c r="Y13" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="Z13" t="s">
         <v>236</v>
       </c>
       <c r="AA13">
-        <v>0.99797437485078455</v>
+        <v>0.99727051178070425</v>
       </c>
       <c r="AB13">
-        <v>37.136461068950517</v>
+        <v>50.040617353755373</v>
       </c>
       <c r="AD13" t="s">
         <v>209</v>
@@ -6176,13 +6176,13 @@
         <v>258</v>
       </c>
       <c r="AN13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AO13">
-        <v>0.99763776609661003</v>
+        <v>0.9927360267512606</v>
       </c>
       <c r="AP13">
-        <v>43.307621562148476</v>
+        <v>133.17284289355615</v>
       </c>
     </row>
     <row r="14" spans="2:42">
@@ -6247,16 +6247,16 @@
         <v>218</v>
       </c>
       <c r="Y14" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="Z14" t="s">
         <v>237</v>
       </c>
       <c r="AA14">
-        <v>0.998201681747511</v>
+        <v>0.99510391360728279</v>
       </c>
       <c r="AB14">
-        <v>32.969167962298094</v>
+        <v>89.761583866481658</v>
       </c>
       <c r="AD14" t="s">
         <v>209</v>
@@ -6286,13 +6286,13 @@
         <v>259</v>
       </c>
       <c r="AN14" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="AO14">
-        <v>0.9927360267512606</v>
+        <v>0.99545389931512118</v>
       </c>
       <c r="AP14">
-        <v>133.17284289355615</v>
+        <v>83.345179222779151</v>
       </c>
     </row>
     <row r="15" spans="2:42">
@@ -6357,16 +6357,16 @@
         <v>220</v>
       </c>
       <c r="Y15" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="Z15" t="s">
         <v>238</v>
       </c>
       <c r="AA15">
-        <v>0.98763915166972838</v>
+        <v>0.99483713382754202</v>
       </c>
       <c r="AB15">
-        <v>226.61555272164699</v>
+        <v>94.652546495062282</v>
       </c>
       <c r="AD15" t="s">
         <v>209</v>
@@ -6393,16 +6393,16 @@
         <v>252</v>
       </c>
       <c r="AM15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AN15" t="s">
-        <v>261</v>
+        <v>236</v>
       </c>
       <c r="AO15">
-        <v>0.99828324379345523</v>
+        <v>0.99763776609661003</v>
       </c>
       <c r="AP15">
-        <v>31.473863786654263</v>
+        <v>43.307621562148476</v>
       </c>
     </row>
     <row r="16" spans="2:42">
@@ -6467,16 +6467,16 @@
         <v>222</v>
       </c>
       <c r="Y16" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="Z16" t="s">
         <v>239</v>
       </c>
       <c r="AA16">
-        <v>0.9973662353879873</v>
+        <v>0.9966237176926277</v>
       </c>
       <c r="AB16">
-        <v>48.285684553565716</v>
+        <v>61.898508968492948</v>
       </c>
     </row>
     <row r="17" spans="2:28">
@@ -6541,16 +6541,16 @@
         <v>224</v>
       </c>
       <c r="Y17" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="Z17" t="s">
         <v>240</v>
       </c>
       <c r="AA17">
-        <v>0.99508741713487281</v>
+        <v>0.99797437485078455</v>
       </c>
       <c r="AB17">
-        <v>90.064019193998561</v>
+        <v>37.136461068950517</v>
       </c>
     </row>
     <row r="18" spans="2:28">
@@ -6615,16 +6615,16 @@
         <v>226</v>
       </c>
       <c r="Y18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Z18" t="s">
         <v>241</v>
       </c>
       <c r="AA18">
-        <v>0.99510391360728279</v>
+        <v>0.9973662353879873</v>
       </c>
       <c r="AB18">
-        <v>89.761583866481658</v>
+        <v>48.285684553565716</v>
       </c>
     </row>
     <row r="19" spans="2:28">
@@ -6689,16 +6689,16 @@
         <v>228</v>
       </c>
       <c r="Y19" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="Z19" t="s">
         <v>242</v>
       </c>
       <c r="AA19">
-        <v>0.99559026704960707</v>
+        <v>0.99508741713487281</v>
       </c>
       <c r="AB19">
-        <v>80.845104090536353</v>
+        <v>90.064019193998561</v>
       </c>
     </row>
     <row r="20" spans="2:28">
@@ -6763,16 +6763,16 @@
         <v>230</v>
       </c>
       <c r="Y20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Z20" t="s">
         <v>243</v>
       </c>
       <c r="AA20">
-        <v>0.99727051178070425</v>
+        <v>0.98763915166972838</v>
       </c>
       <c r="AB20">
-        <v>50.040617353755373</v>
+        <v>226.61555272164699</v>
       </c>
     </row>
   </sheetData>
@@ -6781,7 +6781,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F685A0A5-7E95-4D42-84DB-CC8F3801B256}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC6AA589-B14B-404A-AF5C-4422A1A13A8E}">
   <dimension ref="B9:M15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6854,7 +6854,7 @@
         <v>262</v>
       </c>
       <c r="K11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="L11">
         <v>1.2897218124341414</v>
@@ -6889,7 +6889,7 @@
         <v>264</v>
       </c>
       <c r="K12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="L12">
         <v>0.28038164602463972</v>
@@ -6924,7 +6924,7 @@
         <v>266</v>
       </c>
       <c r="K13" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="L13">
         <v>1.2619807953067491E-2</v>
@@ -6959,7 +6959,7 @@
         <v>268</v>
       </c>
       <c r="K14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="L14">
         <v>0.43107241214667685</v>
@@ -6994,7 +6994,7 @@
         <v>270</v>
       </c>
       <c r="K15" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="L15">
         <v>0.22221482050297564</v>
@@ -7009,7 +7009,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87773F4C-678B-4309-BEC1-C5C693AD9153}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{296F6950-72F5-495C-93D8-70377E313EE5}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>